<commit_message>
Update CN 296 -> 299
</commit_message>
<xml_diff>
--- a/dashboard/autogen/CN296_301.xlsx
+++ b/dashboard/autogen/CN296_301.xlsx
@@ -32,12 +32,10 @@
     </font>
     <font>
       <name val="Times New Roman"/>
-      <color indexed="64"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color indexed="64"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -80,31 +78,31 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
         <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -112,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -146,6 +144,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -480,16 +481,20 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>report_medical_records_service (rms)</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
- Lượt xét nghiệm: Đếm tổng số bản ghi có rms.ma_nhom_dich_vu_report = 9 và có cùng rms.thoi_gian
- Năm sử dụng dịch vụ: rms.thoi_gian (Year)
- Tháng sử dụng dịch vụ: rms.thoi_gian (Month)
- Cơ sở khám chữa bệnh: rms.ten_csyt</t>
+          <t>medical_records_services (mrs)
+ medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
+ cats_services_groups_reports_details (srd) (mrs.service_code = srd.service_code_vi)
+ cats_services_groups_reports (sr) (srd.service_group_id = sr.service_group_id)
+ Điều kiện: mrs.is_delete = 0; mr.is_delete = 0; srd.is_delete = 0, srd.is_active = 1; sr.is_delete = 0, sr.is_active = 1</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Tháng thực hiện: MONTH(mrs.decision_date)
+ Lượt xét nghiệm: Đếm số bản ghi mrs không trùng (COUNT DISTINCT mrs.record_service_id) có sr.code_vi IN ('9','22', '23', '24', '25', 'XNK') và có cùng ngày mrs.decision_date
+ Năm thực hiện: YEAR(mrs.decision_date)
+ Tháng thực hiện: MONTH(mrs.decision_date)
+ Cơ sở khám chữa bệnh: mr.healthfacilities_id</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
@@ -501,10 +506,10 @@
         <is>
           <t>SELECT nam,
        thang,
-       SUM(so_luot) AS luot_xet_nghiem
+       COUNT(DISTINCT id_dich_vu) AS luot_xet_nghiem
 FROM emr_db_tong_hop_cls
 WHERE ma_csyt = :ma_csyt
-  AND ma_nhom = '9'
+  AND ma_nhom IN ('9', '22', '23', '24', '25', 'XNK')
   AND ngay_thuc_hien &gt;= :from_date
   AND ngay_thuc_hien &lt; :to_date
   AND (:thang IS NULL OR thang = :thang)
@@ -526,16 +531,20 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>report_medical_records_service (rms)</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
- Lượt siêu âm: Đếm tổng số bản ghi có rms.ma_nhom_dich_vu_report = 6, 7, 8 và có cùng rms.thoi_gian
- Năm sử dụng dịch vụ: rms.thoi_gian (Year)
- Tháng sử dụng dịch vụ: rms.thoi_gian (Month)
- Cơ sở khám chữa bệnh: rms.ten_csyt</t>
+          <t>medical_records_services (mrs)
+ medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
+cats_services_groups_reports_details (srd) (mrs.service_code = srd.service_code_vi)
+cats_services_groups_reports (sr) (srd.service_group_id = sr.service_group_id)
+ Điều kiện: mrs.is_delete = 0; mr.is_delete = 0; srd.is_delete = 0, srd.is_active = 1; sr.is_delete = 0, sr.is_active = 1</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Tháng thực hiện: MONTH(mrs.decision_date)
+ Lượt siêu âm: Đếm số bản ghi mrs không trùng (COUNT DISTINCT mrs.record_service_id) có sr.code_vi IN ('('6, 7, 8, '18Sieuam')') và có cùng ngày mrs.decision_date
+ Năm thực hiện: YEAR(mrs.decision_date)
+ Tháng thực hiện: MONTH(mrs.decision_date)
+ Cơ sở khám chữa bệnh: mr.healthfacilities_id</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -547,10 +556,10 @@
         <is>
           <t>SELECT nam,
        thang,
-       SUM(so_luot) AS luot_sieu_am
+       COUNT(DISTINCT id_dich_vu) AS luot_sieu_am
 FROM emr_db_tong_hop_cls
 WHERE ma_csyt = :ma_csyt
-  AND ma_nhom IN ('6', '7', '8')
+  AND ma_nhom IN ('6', '7', '8', '18Sieuam')
   AND ngay_thuc_hien &gt;= :from_date
   AND ngay_thuc_hien &lt; :to_date
   AND (:thang IS NULL OR thang = :thang)
@@ -572,16 +581,20 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>report_medical_records_service (rms)</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
- Lượt chụp X-quang: Đếm tổng số bản ghi có rms.ma_nhom_dich_vu_report = 1, 2 và có cùng rms.thoi_gian
- Năm sử dụng dịch vụ: rms.thoi_gian (Year)
- Tháng sử dụng dịch vụ: rms.thoi_gian (Month)
- Cơ sở khám chữa bệnh: rms.ten_csyt</t>
+          <t>medical_records_services (mrs)
+ medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
+ cats_services_groups_reports_details (srd) (mrs.service_code = srd.service_code_vi)
+cats_services_groups_reports (sr) (srd.service_group_id = sr.service_group_id)
+ Điều kiện: mrs.is_delete = 0; mr.is_delete = 0; srd.is_delete = 0, srd.is_active = 1; sr.is_delete = 0, sr.is_active = 1</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Tháng thực hiện: MONTH(mrs.decision_date)
+ Lượt chụp X-quang: Đếm số bản ghi mrs không trùng (COUNT DISTINCT mrs.record_service_id) có sr.code_vi IN 1,2,'18Xquang') và có cùng ngày mrs.decision_date
+ Năm thực hiện: YEAR(mrs.decision_date)
+ Tháng thực hiện: MONTH(mrs.decision_date)
+ Cơ sở khám chữa bệnh: mr.healthfacilities_id</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -593,10 +606,10 @@
         <is>
           <t>SELECT nam,
        thang,
-       SUM(so_luot) AS luot_xquang
+       COUNT(DISTINCT id_dich_vu) AS luot_xquang
 FROM emr_db_tong_hop_cls
 WHERE ma_csyt = :ma_csyt
-  AND ma_nhom IN ('1', '2')
+  AND ma_nhom IN ('1', '2', '18Xquang')
   AND ngay_thuc_hien &gt;= :from_date
   AND ngay_thuc_hien &lt; :to_date
   AND (:thang IS NULL OR thang = :thang)
@@ -618,16 +631,20 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>report_medical_records_service (rms)</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
- Lượt chụp CT/MRI: Đếm tổng số bản ghi có rms.ma_nhom_dich_vu_report = 3, 4, 5 và có cùng rms.thoi_gian
- Năm sử dụng dịch vụ: rms.thoi_gian (Year)
- Tháng sử dụng dịch vụ: rms.thoi_gian (Month)
- Cơ sở khám chữa bệnh: rms.ten_csyt</t>
+          <t>medical_records_services (mrs)
+ medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
+ cats_services_groups_reports_details (srd) (mrs.service_code = srd.service_code_vi)
+ cats_services_groups_reports (sr) (srd.service_group_id = sr.service_group_id)
+ Điều kiện: mrs.is_delete = 0; mr.is_delete = 0; srd.is_delete = 0, srd.is_active = 1; sr.is_delete = 0, sr.is_active = 1</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Tháng thực hiện: MONTH(mrs.decision_date)
+ Lượt chụp CT/MRI: Đếm số bản ghi mrs không trùng (COUNT DISTINCT mrs.record_service_id) có sr.code_vi IN ((3,4,5'18CTS', '18MRI')') và có cùng ngày mrs.decision_date
+ Năm thực hiện: YEAR(mrs.decision_date)
+ Tháng thực hiện: MONTH(mrs.decision_date)
+ Cơ sở khám chữa bệnh: mr.healthfacilities_id</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -639,10 +656,10 @@
         <is>
           <t>SELECT nam,
        thang,
-       SUM(so_luot) AS luot_ct_mri
+       COUNT(DISTINCT id_dich_vu) AS luot_ct_mri
 FROM emr_db_tong_hop_cls
 WHERE ma_csyt = :ma_csyt
-  AND ma_nhom IN ('3', '4', '5')
+  AND ma_nhom IN ('3', '4', '5', '18CTS', '18MRI')
   AND ngay_thuc_hien &gt;= :from_date
   AND ngay_thuc_hien &lt; :to_date
   AND (:thang IS NULL OR thang = :thang)
@@ -662,14 +679,14 @@
           <t>Biểu đồ số ca phẫu thuật tại bệnh viện theo thời gian</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>medical_records_services (mrs)
  medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
  cats_cost_groups (ccg) (mrs.cost_group_id = ccg.cost_group_id)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Ngày y lệnh: mrs.decision_date
  CSKCB: mrs.healthfacilities_id
@@ -710,14 +727,14 @@
           <t>Biểu đồ số ca thủ thuật tại bệnh viện theo thời gian</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>medical_records_services (mrs)
  medical_records (mr) (mrs.medical_record_id = mr.medical_record_id)
  cats_cost_groups (ccg) (mrs.cost_group_id = ccg.cost_group_id)</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Ngày y lệnh: mrs.decision_date
  CSKCB: mrs.healthfacilities_id

</xml_diff>